<commit_message>
Add standalone SQL perf pipeline, Streamlit explorer, analysis scripts, and refreshed artifacts/reports
- Include standalone_sql_perf_pipeline (training, regression, schema stats, figures)
- Add sql_query_explorer Streamlit app and supporting utilities
- Refresh model artifacts, datasets, and report outputs
- Extend markdown documentation and narrative figures
- Ignore Office lock files (~$*) in .gitignore
- Remove tracked SQLite WAL/SHM sidecar files for card_games

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/markdowns/ADVANCED MML BREIFS/COM 763 Portfolio Task 1 Marking Rubric.xlsx
+++ b/markdowns/ADVANCED MML BREIFS/COM 763 Portfolio Task 1 Marking Rubric.xlsx
@@ -1,37 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29825"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{39A7C2C8-6B0B-48CF-8ABE-DE8ECCFD3094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aled_\Downloads\COM763---ML-pipeline-for-SQL-error-detection-project\markdowns\ADVANCED MML BREIFS\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7447E1DB-A920-4A72-9D88-8676BBD0BAA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="16200" windowHeight="9308" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Weighting</t>
   </si>
@@ -39,24 +33,6 @@
     <t>Section Title</t>
   </si>
   <si>
-    <t>0% (Non-submission)</t>
-  </si>
-  <si>
-    <t>1–29% Unsatisfactory</t>
-  </si>
-  <si>
-    <t>30–39% Minimum</t>
-  </si>
-  <si>
-    <t>40–49% Satisfactory</t>
-  </si>
-  <si>
-    <t>50–59% Good</t>
-  </si>
-  <si>
-    <t>60–69% Very Good</t>
-  </si>
-  <si>
     <t>70–79% Excellent</t>
   </si>
   <si>
@@ -69,24 +45,6 @@
     <t>Problem Definition and System Framing</t>
   </si>
   <si>
-    <t>No submission</t>
-  </si>
-  <si>
-    <t>Fails to define a problem or justify ML use.</t>
-  </si>
-  <si>
-    <t>Poorly defined problem with little justification for ML.</t>
-  </si>
-  <si>
-    <t>Basic definition; justification for ML is present but lacks depth.</t>
-  </si>
-  <si>
-    <t>Clear definition of a real-world problem and logical ML justification.</t>
-  </si>
-  <si>
-    <t>Strong framing; detailed task formulation and clear rationale.</t>
-  </si>
-  <si>
     <t>Excellent framing with deep insight into the problem context.</t>
   </si>
   <si>
@@ -99,21 +57,6 @@
     <t>Data Pipeline and Feature Handling</t>
   </si>
   <si>
-    <t>No description of data preparation or handling.</t>
-  </si>
-  <si>
-    <t>Minimal data handling; lack of justification for transformations.</t>
-  </si>
-  <si>
-    <t>Basic data preparation; transformations mentioned but not well-justified.</t>
-  </si>
-  <si>
-    <t>Clear description of the pipeline; most feature choices are justified.</t>
-  </si>
-  <si>
-    <t>High-quality data handling; detailed justification of all steps.</t>
-  </si>
-  <si>
     <t>Strong engineering practice in data processing and feature engineering.</t>
   </si>
   <si>
@@ -126,21 +69,6 @@
     <t>Model Implementation and Debugging</t>
   </si>
   <si>
-    <t>No evidence of implementation or debugging.</t>
-  </si>
-  <si>
-    <t>Poor implementation; no evidence of iterative improvement.</t>
-  </si>
-  <si>
-    <t>Basic implementation; minimal evidence of debugging or design logic.</t>
-  </si>
-  <si>
-    <t>Solid implementation; some evidence of debugging and design choices.</t>
-  </si>
-  <si>
-    <t>Strong implementation; clear evidence of iterative improvement.</t>
-  </si>
-  <si>
     <t>Expert implementation; rigorous debugging and clear design logic.</t>
   </si>
   <si>
@@ -153,21 +81,6 @@
     <t>Experimental Evaluation and Model Selection</t>
   </si>
   <si>
-    <t>Lacks evaluation or comparison of models.</t>
-  </si>
-  <si>
-    <t>Minimal evaluation; poor choice of metrics or comparison logic.</t>
-  </si>
-  <si>
-    <t>Basic evaluation using relevant metrics; some comparison present.</t>
-  </si>
-  <si>
-    <t>Good evaluation; comparison of models is logical and evidenced.</t>
-  </si>
-  <si>
-    <t>Rigorous evaluation; strong justification for final model selection.</t>
-  </si>
-  <si>
     <t>Excellent rigor; deep comparison using appropriate, diverse metrics.</t>
   </si>
   <si>
@@ -178,21 +91,6 @@
   </si>
   <si>
     <t>Presentation, Structure &amp; Communication</t>
-  </si>
-  <si>
-    <t>Unstructured; lacks required visuals and screenshots.</t>
-  </si>
-  <si>
-    <t>Poorly organized; minimal visuals; lacks professionalism.</t>
-  </si>
-  <si>
-    <t>Adequate structure; includes basic screenshots and visuals.</t>
-  </si>
-  <si>
-    <t>Clear organization; good quality visuals and implementation screenshots.</t>
-  </si>
-  <si>
-    <t>Very professional; well-structured with high-quality visual evidence.</t>
   </si>
   <si>
     <t>Excellent professionalism; seamless narrative and clear visual data.</t>
@@ -208,7 +106,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -229,12 +127,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
     </font>
     <font>
       <sz val="10"/>
@@ -277,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -288,23 +180,13 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -642,24 +524,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultColWidth="17.5703125" defaultRowHeight="70.5" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="17.59765625" defaultRowHeight="70.5" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="17.5703125" style="1"/>
-    <col min="3" max="3" width="17.5703125" style="10"/>
-    <col min="4" max="11" width="17.5703125" style="1"/>
-    <col min="12" max="12" width="17.5703125" style="5"/>
-    <col min="13" max="13" width="17.5703125" style="1"/>
-    <col min="14" max="16384" width="17.5703125" style="4"/>
+    <col min="1" max="2" width="17.59765625" style="1"/>
+    <col min="3" max="3" width="17.59765625" style="6"/>
+    <col min="4" max="13" width="17.59765625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="70.5" customHeight="1">
+    <row r="1" spans="1:13" ht="70.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -668,204 +547,132 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="H1"/>
+      <c r="I1"/>
+      <c r="J1"/>
+      <c r="K1"/>
+      <c r="L1"/>
+      <c r="M1"/>
     </row>
-    <row r="2" spans="1:12" ht="70.5" customHeight="1">
+    <row r="2" spans="1:13" ht="70.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="3">
         <v>0.15</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="L2" s="6"/>
+        <v>5</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="4"/>
+      <c r="H2"/>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2"/>
     </row>
-    <row r="3" spans="1:12" ht="70.5" customHeight="1">
+    <row r="3" spans="1:13" ht="70.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="3">
         <v>0.25</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="L3" s="6"/>
+      <c r="F3" s="4"/>
+      <c r="H3"/>
+      <c r="I3"/>
+      <c r="J3"/>
+      <c r="K3"/>
+      <c r="L3"/>
+      <c r="M3"/>
     </row>
-    <row r="4" spans="1:12" ht="70.5" customHeight="1">
+    <row r="4" spans="1:13" ht="70.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="3">
         <v>0.3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="L4" s="6"/>
+        <v>13</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4"/>
+      <c r="K4"/>
+      <c r="L4"/>
+      <c r="M4"/>
     </row>
-    <row r="5" spans="1:12" ht="70.5" customHeight="1">
+    <row r="5" spans="1:13" ht="70.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="3">
         <v>0.2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="L5" s="6"/>
+        <v>17</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="4"/>
+      <c r="H5"/>
+      <c r="I5"/>
+      <c r="J5"/>
+      <c r="K5"/>
+      <c r="L5"/>
+      <c r="M5"/>
     </row>
-    <row r="6" spans="1:12" ht="70.5" customHeight="1">
+    <row r="6" spans="1:13" ht="70.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="3">
         <v>0.1</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="L6" s="6"/>
+        <v>21</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="4"/>
+      <c r="H6"/>
+      <c r="I6"/>
+      <c r="J6"/>
+      <c r="K6"/>
+      <c r="L6"/>
+      <c r="M6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -873,15 +680,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A2B77D17EB858E4BB4FFA17E28B4173A" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="49fa6669263639da42240932e5eee154">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="5418a382-16e9-4b6e-9216-45c260aed3cc" xmlns:ns3="f51a6981-c302-436e-80b4-016e68f513fa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d7f3d36a0250d6d1aed1872588b57564" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1099,6 +897,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1113,13 +920,41 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F16E39E-8DD4-4B06-ABB1-222FB9E85D90}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C307795-5BFE-4306-9BD1-629E965821D3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="5418a382-16e9-4b6e-9216-45c260aed3cc"/>
+    <ds:schemaRef ds:uri="f51a6981-c302-436e-80b4-016e68f513fa"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C307795-5BFE-4306-9BD1-629E965821D3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F16E39E-8DD4-4B06-ABB1-222FB9E85D90}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{676E5EF3-8068-41AC-9868-CC14C0B8E58D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{676E5EF3-8068-41AC-9868-CC14C0B8E58D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="f51a6981-c302-436e-80b4-016e68f513fa"/>
+    <ds:schemaRef ds:uri="5418a382-16e9-4b6e-9216-45c260aed3cc"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>